<commit_message>
Pin exact dropdown options and submit button from the live form
The probe reached the English form and returned every dropdown's real options.
Bake them into the template Lists and wire the two that were still free text:
- Level Test: "Y : I will participate…" / "N : I agree to start directly…"
- Pre-Korean Class: "Yes (will automatically be assigned to level 1…)" / "No"
- Tuition Payment: "Account Number" / "Flywire"
- Purpose of Study: To Enter University / Hobby / TOPIK test / Find Job in Korea /
  Find Job in other Country / Other
- Estimated Period: 3 months / 6 months / 9 months / 1 year / 1~2 years / 2 years
- VISA status: B-1 … No Visa (new dropdown)
- Preferred Language order English/Chinese/Japanese/Korean

Set HY_SUBMIT_TEXT default to "Save & Submit" (the real submit button).
Nationality still a short list pending the full set from form.html.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TvNm7wqFpsjRLmFD875nU
</commit_message>
<xml_diff>
--- a/hanyang-apply-bot/Hanyang_Students_Template.xlsx
+++ b/hanyang-apply-bot/Hanyang_Students_Template.xlsx
@@ -341,16 +341,6 @@
         <t>1–8.</t>
       </text>
     </comment>
-    <comment ref="F2" authorId="0" shapeId="0">
-      <text>
-        <t>CONFIRM exact wording.</t>
-      </text>
-    </comment>
-    <comment ref="I2" authorId="0" shapeId="0">
-      <text>
-        <t>CONFIRM options.</t>
-      </text>
-    </comment>
     <comment ref="J2" authorId="0" shapeId="0">
       <text>
         <t>Folder under uploads/ with photo.jpg, passport.jpg, education.pdf, gap.pdf, financial.pdf, family.pdf, other.pdf. Keep format e.g. NN_FAMILY_GIVEN.</t>
@@ -418,7 +408,7 @@
     </comment>
     <comment ref="AE2" authorId="0" shapeId="0">
       <text>
-        <t>Only if they already hold a visa. CONFIRM.</t>
+        <t>Only if they already hold a visa.</t>
       </text>
     </comment>
     <comment ref="AG2" authorId="0" shapeId="0">
@@ -434,16 +424,6 @@
     <comment ref="AJ2" authorId="0" shapeId="0">
       <text>
         <t>e.g. 2022-01 ~ 2022-06.</t>
-      </text>
-    </comment>
-    <comment ref="AM2" authorId="0" shapeId="0">
-      <text>
-        <t>CONFIRM options.</t>
-      </text>
-    </comment>
-    <comment ref="AO2" authorId="0" shapeId="0">
-      <text>
-        <t>CONFIRM options.</t>
       </text>
     </comment>
     <comment ref="AS2" authorId="0" shapeId="0">
@@ -754,7 +734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -950,7 +930,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Participate | Don't participate (direct placement into Level 1)</t>
+          <t>Y : I will participate in the offline level test | N : I agree to start directly with Level 1 classes without taking the level test</t>
         </is>
       </c>
     </row>
@@ -969,120 +949,144 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Payment</t>
+          <t>PreKorean</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Lump-sum payment | Installment</t>
+          <t>Yes (will automatically be assigned to level 1 without level test) | No</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Payment</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Male | Female</t>
+          <t>Account Number | Flywire</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Education</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Undergraduate | Postgraduate or Higher | High School</t>
+          <t>Male | Female</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>Education</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Enter a university | Employment | Interest / Culture | Others</t>
+          <t>Undergraduate | Postgraduate or Higher | High School</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>AimLevel</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Level 1 | Level 2 | Level 3 | Level 4 | Level 5 | Level 6</t>
+          <t>To Enter University | Hobby | TOPIK test | Find Job in Korea | Find Job in other Country | Other</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>EstPeriod</t>
+          <t>AimLevel</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>1 semester | 2 semesters | 3 semesters | 4 semesters</t>
+          <t>Level 1 | Level 2 | Level 3 | Level 4 | Level 5 | Level 6</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>PrefLanguage</t>
+          <t>EstPeriod</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Korean | English | Chinese | Japanese | Others</t>
+          <t>3 months | 6 months | 9 months | 1 year | 1~2 years | 2 years</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Messenger</t>
+          <t>PrefLanguage</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Kakao | Wechat | Line</t>
+          <t>English | Chinese | Japanese | Korean</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>YesBlank</t>
+          <t>Messenger</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>Kakao | Wechat | Line</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>YesBlank</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>VisaStatus</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>B-1 | B-2 | C-2 | C-3 | C-6 | D-1 | D-2 | D-4 | D-6 | D-8 | E-1 | E-2 | E-3 | E-6 | E-7 | E-9 | F-1 | F-2 | F-3 | F-4 | F-5 | F-6 | H-1 | H-2 | No Visa</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>Nationality</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Bangladesh | India | Pakistan | Nepal | Sri Lanka | Bhutan | Vietnam | China | Indonesia | Uzbekistan | Mongolia | Myanmar | Philippines | Thailand | Japan | Others</t>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Bangladesh | India | Pakistan | Nepal | Srilanka | Bhutan | Vietnam | China | Indonesia | Uzbekistan | Mongolia | Myanmar | Philippines | Thailand | Japan</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1122,6 +1126,8 @@
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="30" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1147,50 +1153,60 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
+          <t>PreKorean</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Education</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>AimLevel</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>EstPeriod</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>PrefLanguage</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>Messenger</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>YesBlank</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>VisaStatus</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Nationality</t>
         </is>
@@ -1209,7 +1225,7 @@
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>Participate</t>
+          <t>Y : I will participate in the offline level test</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
@@ -1219,50 +1235,60 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Lump-sum payment</t>
+          <t>Yes (will automatically be assigned to level 1 without level test)</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
+          <t>Account Number</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
           <t>Male</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Undergraduate</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>Enter a university</t>
-        </is>
-      </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
+          <t>To Enter University</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
           <t>Level 1</t>
         </is>
       </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>1 semester</t>
-        </is>
-      </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>3 months</t>
         </is>
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
           <t>Kakao</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
+        <is>
+          <t>B-1</t>
+        </is>
+      </c>
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>Bangladesh</t>
         </is>
@@ -1281,7 +1307,7 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Don't participate (direct placement into Level 1)</t>
+          <t>N : I agree to start directly with Level 1 classes without taking the level test</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1291,45 +1317,55 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Installment</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
+          <t>Flywire</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
           <t>Female</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Postgraduate or Higher</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>Employment</t>
-        </is>
-      </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
+          <t>Hobby</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
           <t>Level 2</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
-        <is>
-          <t>2 semesters</t>
-        </is>
-      </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>6 months</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
+          <t>Chinese</t>
+        </is>
+      </c>
+      <c r="M3" s="6" t="inlineStr">
+        <is>
           <t>Wechat</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>B-2</t>
+        </is>
+      </c>
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>India</t>
         </is>
@@ -1346,37 +1382,42 @@
           <t>Don't Mind (Automatically assigned to the afternoon half.)</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>High School</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Interest / Culture</t>
-        </is>
-      </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
+          <t>TOPIK test</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
           <t>Level 3</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>3 semesters</t>
-        </is>
-      </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>Chinese</t>
+          <t>9 months</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="M4" s="6" t="inlineStr">
+        <is>
           <t>Line</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
+        <is>
+          <t>C-2</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>Pakistan</t>
         </is>
@@ -1388,27 +1429,32 @@
           <t>4</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Others</t>
-        </is>
-      </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
+          <t>Find Job in Korea</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
           <t>Level 4</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>4 semesters</t>
-        </is>
-      </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Japanese</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
+          <t>1 year</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Korean</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>C-3</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>Nepal</t>
         </is>
@@ -1422,17 +1468,27 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
+          <t>Find Job in other Country</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
           <t>Level 5</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Others</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>Sri Lanka</t>
+          <t>1~2 years</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>C-6</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>Srilanka</t>
         </is>
       </c>
     </row>
@@ -1444,10 +1500,25 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
           <t>Level 6</t>
         </is>
       </c>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>2 years</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr">
+        <is>
+          <t>D-1</t>
+        </is>
+      </c>
+      <c r="P7" s="6" t="inlineStr">
         <is>
           <t>Bhutan</t>
         </is>
@@ -1459,7 +1530,12 @@
           <t>7</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
+        <is>
+          <t>D-2</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>Vietnam</t>
         </is>
@@ -1471,65 +1547,168 @@
           <t>8</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="O9" s="6" t="inlineStr">
+        <is>
+          <t>D-4</t>
+        </is>
+      </c>
+      <c r="P9" s="6" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="N10" s="6" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
+        <is>
+          <t>D-6</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="inlineStr">
         <is>
           <t>Indonesia</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="N11" s="6" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
+        <is>
+          <t>D-8</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
         <is>
           <t>Uzbekistan</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="N12" s="6" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>E-1</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr">
         <is>
           <t>Mongolia</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="N13" s="6" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
+        <is>
+          <t>E-2</t>
+        </is>
+      </c>
+      <c r="P13" s="6" t="inlineStr">
         <is>
           <t>Myanmar</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="N14" s="6" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
+        <is>
+          <t>E-3</t>
+        </is>
+      </c>
+      <c r="P14" s="6" t="inlineStr">
         <is>
           <t>Philippines</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="N15" s="6" t="inlineStr">
+      <c r="O15" s="6" t="inlineStr">
+        <is>
+          <t>E-6</t>
+        </is>
+      </c>
+      <c r="P15" s="6" t="inlineStr">
         <is>
           <t>Thailand</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="N16" s="6" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>E-7</t>
+        </is>
+      </c>
+      <c r="P16" s="6" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="N17" s="6" t="inlineStr">
-        <is>
-          <t>Others</t>
+      <c r="O17" s="6" t="inlineStr">
+        <is>
+          <t>E-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="O18" s="6" t="inlineStr">
+        <is>
+          <t>F-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="O19" s="6" t="inlineStr">
+        <is>
+          <t>F-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="O20" s="6" t="inlineStr">
+        <is>
+          <t>F-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="O21" s="6" t="inlineStr">
+        <is>
+          <t>F-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="O22" s="6" t="inlineStr">
+        <is>
+          <t>F-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="O23" s="6" t="inlineStr">
+        <is>
+          <t>F-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="O24" s="6" t="inlineStr">
+        <is>
+          <t>H-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="O25" s="6" t="inlineStr">
+        <is>
+          <t>H-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="O26" s="6" t="inlineStr">
+        <is>
+          <t>No Visa</t>
         </is>
       </c>
     </row>
@@ -1552,10 +1731,10 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
@@ -1925,7 +2104,7 @@
       </c>
       <c r="F3" s="19" t="inlineStr">
         <is>
-          <t>Don't participate (direct placement into Level 1)</t>
+          <t>N : I agree to start directly with Level 1 classes without taking the level test</t>
         </is>
       </c>
       <c r="G3" s="19" t="inlineStr">
@@ -1940,7 +2119,7 @@
       </c>
       <c r="I3" s="19" t="inlineStr">
         <is>
-          <t>Lump-sum payment</t>
+          <t>Account Number</t>
         </is>
       </c>
       <c r="J3" s="19" t="inlineStr">
@@ -2050,7 +2229,7 @@
       <c r="AL3" s="19" t="inlineStr"/>
       <c r="AM3" s="19" t="inlineStr">
         <is>
-          <t>Enter a university</t>
+          <t>To Enter University</t>
         </is>
       </c>
       <c r="AN3" s="19" t="inlineStr">
@@ -2060,7 +2239,7 @@
       </c>
       <c r="AO3" s="19" t="inlineStr">
         <is>
-          <t>2 semesters</t>
+          <t>1 year</t>
         </is>
       </c>
       <c r="AP3" s="19" t="inlineStr">
@@ -5942,7 +6121,7 @@
     <mergeCell ref="AD1:AG1"/>
     <mergeCell ref="D1:I1"/>
   </mergeCells>
-  <dataValidations count="16">
+  <dataValidations count="17">
     <dataValidation sqref="D3:D78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
       <formula1>Lists!$A$2:$A$9</formula1>
     </dataValidation>
@@ -5953,43 +6132,46 @@
       <formula1>Lists!$C$2:$C$3</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$D$2:$D$3</formula1>
+      <formula1>Lists!$E$2:$E$3</formula1>
     </dataValidation>
     <dataValidation sqref="H3:H78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
       <formula1>Lists!$D$2:$D$3</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$E$2:$E$3</formula1>
+      <formula1>Lists!$F$2:$F$3</formula1>
     </dataValidation>
     <dataValidation sqref="N3:N78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$F$2:$F$3</formula1>
+      <formula1>Lists!$G$2:$G$3</formula1>
     </dataValidation>
     <dataValidation sqref="R3:R78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$M$2:$M$2</formula1>
+      <formula1>Lists!$N$2:$N$2</formula1>
     </dataValidation>
     <dataValidation sqref="V3:V78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$L$2:$L$4</formula1>
+      <formula1>Lists!$M$2:$M$4</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$K$2:$K$6</formula1>
+      <formula1>Lists!$L$2:$L$5</formula1>
     </dataValidation>
     <dataValidation sqref="AC3:AC78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$G$2:$G$4</formula1>
+      <formula1>Lists!$H$2:$H$4</formula1>
     </dataValidation>
     <dataValidation sqref="AD3:AD78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
       <formula1>Lists!$D$2:$D$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE3:AE78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
+      <formula1>Lists!$O$2:$O$26</formula1>
     </dataValidation>
     <dataValidation sqref="AH3:AH78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
       <formula1>Lists!$D$2:$D$3</formula1>
     </dataValidation>
     <dataValidation sqref="AM3:AM78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$H$2:$H$5</formula1>
+      <formula1>Lists!$I$2:$I$7</formula1>
     </dataValidation>
     <dataValidation sqref="AN3:AN78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$I$2:$I$7</formula1>
+      <formula1>Lists!$J$2:$J$7</formula1>
     </dataValidation>
     <dataValidation sqref="AO3:AO78" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the dropdown (see the Lists tab)." type="list">
-      <formula1>Lists!$J$2:$J$5</formula1>
+      <formula1>Lists!$K$2:$K$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Handle date cells, keep phone +, tick pledge, select course
From the first live fill test:
- Date of Birth / Date of degree came through as Excel serial numbers (38756,
  46026) because those cells were formatted as dates. The reader now converts a
  date-formatted (serial) or Date cell to YYYY-MM-DD (excelSerialToISO, UTC).
- Excel was stripping the leading "+" from phone numbers. The template now stores
  every data cell as Text (@), so +880/+82, leading zeros and long numbers stay
  verbatim.
- Tick the "Security pledge -> Agree" checkbox before Save & Submit.
- Applying Course radio: fall back to the single visible radio when it is not in
  the labelled row.

Kakao/Wechat/Line left as-is (optional). Self-test 43/43, tsc clean.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013TvNm7wqFpsjRLmFD875nU
</commit_message>
<xml_diff>
--- a/hanyang-apply-bot/Hanyang_Students_Template.xlsx
+++ b/hanyang-apply-bot/Hanyang_Students_Template.xlsx
@@ -235,10 +235,10 @@
     <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="5" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>